<commit_message>
docs: itemize camera/DMS sources + validation logic in API workbook
Three new tabs:
- Camera Sources: 15 state camera networks, adapter family + endpoint,
  with live unit counts pulled from each feed (21,941 cameras)
- DMS + Device Sources: 18 state DMS/arrow-board feeds; 10 keyless ones
  returned 4,601 signs/devices, 8 are key-gated and skipped
- Validation Logic: all 54 coded rules and thresholds across the 7 stages
  (normalize, geometry, DQI, event confidence, the 4 independent
  validators, CWZ 1.0 composition, monitoring)

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KU6vCHVwj8n3HqfggcJ2CP
</commit_message>
<xml_diff>
--- a/docs/Corridor_Communicator_API_Inventory.xlsx
+++ b/docs/Corridor_Communicator_API_Inventory.xlsx
@@ -12,12 +12,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Feed Registry" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External APIs Consumed" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Published Feeds" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DMS + Device Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Logic" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Internal REST API'!$A$1:$I$512</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'State Feed Registry'!$A$1:$G$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'External APIs Consumed'!$A$1:$G$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Published Feeds'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Camera Sources'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DMS + Device Sources'!$A$1:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Validation Logic'!$A$1:$G$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +77,18 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005B6B8C"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008A3A00"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="006B1F8C"/>
     </font>
   </fonts>
   <fills count="4">
@@ -117,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +177,30 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -526,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2105,6 +2147,34 @@
       <c r="A118" t="inlineStr">
         <is>
           <t>Published Feeds - what the platform emits for others to consume</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Camera / DMS / validation tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Camera Sources - 15 state camera networks with live unit counts (pulled 2026-09-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>DMS + Device Sources - 18 state DMS / arrow-board feeds; 8 are key-gated and currently skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Validation Logic - every validation rule and threshold, ingest through CWZ 1.0 composition</t>
         </is>
       </c>
     </row>
@@ -26470,7 +26540,7 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>511 sites for ID, GA, NY, AZ, CA, FL, MN, NC, NV, UT, PA, LA, New England, Austin TX</t>
+          <t>Itemized on the 'Camera Sources' tab - 15 state networks, 21941 cameras</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -26507,7 +26577,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>511/AGOL device endpoints for ID, LA, NJ, NY, WI, ME, AZ, MD, CA, FL, PA, OK, NM, NC, NV, UT, WA</t>
+          <t>Itemized on the 'DMS + Device Sources' tab - 18 state feeds, 4601 signs/devices from the 10 keyless ones</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -27438,4 +27508,3633 @@
   <autoFilter ref="A1:F9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Agency / network</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Adapter family</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Live pull 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Cameras returned</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>With still image</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>https://az511.com/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>644</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>644</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Caltrans CWWP2 (12 districts)</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d&lt;N&gt;/cctv/cctvStatusD&lt;NN&gt;.json</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>3340</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>3340</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>ArcGIS FeatureServer</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_Cameras/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1669</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>1669</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>https://511ga.org/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>4043</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>4043</v>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Idaho</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>https://511.idaho.gov/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>457</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>457</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Iowa</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>ArcGIS FeatureServer</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/8lRhdTsQyJpO52F1/.../Traffic_Cameras_View/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>1252</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>1252</v>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Louisiana</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.511la.org/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>336</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>336</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Maine / New England</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>https://newengland511.org/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>405</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>405</v>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Minnesota</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>CARS cameras_v1</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>https://mntg.carsprogram.org/cameras_v1/api/cameras</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>1528</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>1528</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nvroads.com/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>640</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>640</v>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>511NY getcameras</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>https://511ny.org/api/getcameras?format=json</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>1871</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>1871</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>https://www.drivenc.gov/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.511pa.com/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>1536</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>1536</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Texas (Austin)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Socrata open data</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>https://data.austintexas.gov/resource/b4k4-adkb.json (images: cctv.austinmobility.io)</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>1005</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>1005</v>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Utah</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>IBI/511 cameras (POST)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.udottraffic.utah.gov/ (List/GetData cameras)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>2075</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>2075</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>camera-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr"/>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr"/>
+      <c r="D17" s="17" t="inlineStr"/>
+      <c r="E17" s="17" t="inlineStr"/>
+      <c r="F17" s="17" t="n">
+        <v>21941</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>21941</v>
+      </c>
+      <c r="H17" s="17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Agency</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Adapter family</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Live pull 2026-09-03</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Signs / devices</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Actively displaying</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Portable units</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Key required</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Iowa (DMS corroboration validator)</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>ArcGIS FeatureServer</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/8lRhdTsQyJpO52F1/ArcGIS/rest/services/DMS_View/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>not counted in this pull</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr"/>
+      <c r="H2" s="8" t="inlineStr"/>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Primary DMS source for the DMS validator + device ingest; 10-min cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>https://az511.com/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Caltrans CWWP2 CMS (12 districts)</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d&lt;N&gt;/cms/cmsStatusD&lt;NN&gt;.json</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>1016</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Some districts intermittently 500 and are skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>ArcGIS FeatureServer</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_MessageBoard/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1047</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Fixed DMS with live message text</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Idaho</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>https://511.idaho.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr"/>
+      <c r="H6" s="8" t="inlineStr"/>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Kentucky</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ArcGIS FeatureServer</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>https://services2.arcgis.com/CcI36Pduqd0OR4W9/.../dmsSigns_2020/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Fixed DMS with live message text</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Louisiana</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>https://511la.org/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Maine</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>https://arcgisserver.maine.gov/arcgis/rest/services/mdot/MaineDOT_Dynamic/MapServer/111/query</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Portable = trailer installation type</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Maryland</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer (CHART)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>https://chartimap1.sha.maryland.gov/arcgis/rest/services/CHART/DMS/MapServer/0/query</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>295</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>212</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Route/direction parsed from location string</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nvroads.com/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>https://511nj.org/api/getmessagesigns</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>New Mexico</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Custom REST (NMRoads)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>https://servicev4.nmroads.com/RealMapWAR/GetMessageSigns</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>ERROR: certificate has expired</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>TLS certificate expired as of the pull</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511 (keyless path)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>https://511ny.org/api/getmessagesigns?format=json</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>919</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>919</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>175</v>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Keyless; 175 portable units detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.drivenc.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Oklahoma</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Custom REST (oktraffic.org)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>https://oktraffic.org/api/Devices + /api/DmsStatuses</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>167</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>NTCIP MULTI tags stripped from message text</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>https://gis.penndot.gov/arcgis/rest/services/tsams/tsams/MapServer/17/query</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>962</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Portable = trailer / Type A-B structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Utah</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>https://www.udottraffic.utah.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="8" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>WZDx v4 Device Feed</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>https://wzdx.wsdot.wa.gov/api/v4/DeviceFeed</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Only true WZDx device feed in the set - real arrow boards</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Wisconsin</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>https://511wi.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr"/>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr"/>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL (feeds that returned)</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr"/>
+      <c r="D21" s="18" t="inlineStr"/>
+      <c r="E21" s="18" t="inlineStr"/>
+      <c r="F21" s="18" t="n">
+        <v>4601</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>1789</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <v>429</v>
+      </c>
+      <c r="I21" s="18" t="inlineStr"/>
+      <c r="J21" s="18" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>What it validates</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Rule / threshold as coded</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>On fail</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Output field</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Implemented in</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>0. Ingest / normalize</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Route normalization</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Free-text route strings from 37 different feeds resolve to one canonical route id</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Regex ladder: I-nnn first (ramp strings embed it), then US-nnn, then &lt;ST&gt;-nnn. 'I 380', 'I-380', 'RAMP: I 80E TO 100TH ST' all -&gt; 'I-380'/'I-80'</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Returns null -&gt; the record cannot be route-matched and is skipped by the matcher</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>route / rawRoute</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js normalizeRoute</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>0. Ingest / normalize</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Direction normalization</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Carriageway direction is one of N/S/E/W/BOTH</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>First letter after uppercasing; 'Both'/'B' -&gt; BOTH; anything else -&gt; null (neutral, not a reject)</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>null = unknown, treated as neutral rather than a mismatch</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>direction</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js normalizeDir</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>0. Ingest / normalize</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Coordinate sanity</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Lat/lon are real and not a null-island artifact</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Both finite, not (0,0), |lat| &lt;= 90, |lon| &lt;= 180</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Record dropped at normalize()</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>coordinates</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>device-adapters.js normalize</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>1. Geometry</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Missing content</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Event has geometry and some human content</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>No geometry -&gt; drop. Empty description AND empty location -&gt; drop</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Event filtered out entirely</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>geometry-validator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>1. Geometry</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Fallback-geometry rejection</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Geometry is not an interpolated straight line masquerading as road shape</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>geometrySource in ('straight_line','straight') -&gt; drop</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Event filtered out</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>geometry-validator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>1. Geometry</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>2-point LineString collapse</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>A 2-point line carries no road shape, so it must not render as a road</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>LineString with exactly 2 coordinates -&gt; converted to a Point at the midpoint</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Downgraded to a marker, not dropped</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>_geometryFixed</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>geometry-validator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>1. Geometry</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Curvature test (long lines)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>A very long 'closure' line actually follows the road rather than cutting across it</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>chord &gt; 50 mi AND path length / chord &lt; 1.05 (under 5% curvature) -&gt; drop</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Event filtered out</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>geometry-validator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>1. Geometry</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Type validity</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Point/LineString/Polygon/Multi* are structurally well formed</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Point needs 2 coords; LineString &gt;= 2; Polygon outer ring &gt;= 4; Multi* non-empty; unknown type -&gt; drop</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Event filtered out</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>geometry-validator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Completeness (20%)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Required WZDx fields are actually populated across the feed</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Share of events carrying end time, description, geometry, severity, lanes affected</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Lowers the feed's DQI and letter grade</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>dqi.completeness</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Freshness (15%)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>The feed is being updated and events are not stale</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Update latency + stale-event share</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Lowers DQI</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>dqi.freshness</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy (20%)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Geometry validates and the payload matches schema</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Geometry validation pass rate + schema compliance</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Lowers DQI</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>dqi.accuracy</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Availability (15%)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>The endpoint answers reliably</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Fetch success / failure history per feed key</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Lowers DQI; feeds an outage signal</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>dqi.availability</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js + feed-tracking-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Standardization (15%)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>WZDx compliance, valid event types, ITIS codes</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Share of events using spec-valid enumerations</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Lowers DQI</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>dqi.standardization</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Timeliness (10%)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>No future-dated or long-expired events</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Event age distribution + future-dating check</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Lowers DQI</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>dqi.timeliness</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Usability (5%)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Contact info, restrictions, work-zone type present</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Share of events with actionable detail</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Lowers DQI</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>dqi.usability</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>2. Feed quality (DQI)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Composite + grade</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>One comparable number per state feed</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Weighted mean of the 7 dimensions (weights sum to 1.0) -&gt; letter grade A-F</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Published on the state report cards</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>dqi.overall / grade</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>feed-quality-scorer.js, report-card-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>3. Event confidence</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Completeness (35%)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Per-EVENT (not per-feed) trustworthiness: are the critical fields there</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>id, eventType, start time, finite non-zero lat/lng, and the rest of the critical field set</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Lowers the event's 0-100 score</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>confidence.score</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>event-confidence.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>3. Event confidence</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Geospatial precision (15%)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Point coordinates AND real linestring geometry present</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Both lat/lng and a LineString score full credit</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Lowers score</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>confidence.score</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>event-confidence.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>3. Event confidence</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Temporal validity (20%)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Has a start, has an end, is not stale</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>startTime present, end time present, age within bounds</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Lowers score</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>confidence.score</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>event-confidence.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>3. Event confidence</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Description quality (15%)</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>The narrative is specific, not boilerplate</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Length / specificity heuristic on the description</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Lowers score</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>confidence.score</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>event-confidence.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>3. Event confidence</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Verification (15%)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>DOT operator comments corroborate the record</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Presence of corroborating operator narrative</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Lowers score</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>confidence.score</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>event-confidence.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>3. Event confidence</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Level banding</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Score becomes an operator-facing label</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED &gt;= 85, HIGH 70-84, MEDIUM 50-69, LOW 30-49, UNVERIFIED &lt; 30</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Drives downstream filtering and display</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>confidence.level</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>event-confidence.js levelFromScore</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Gate 1: route</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>The arrow board / portable DMS is on the same route as the zone</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Device route must equal the zone's normalized route. A route-LESS device is allowed through on the other gates but starts at 30 base credit instead of 40</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Return null - not a match</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>x_cwz_connected</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js scoreMatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Gate 2: carriageway</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>The device is not on the opposite side of a divided highway</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Same direction = +25; either side BOTH = +12; opposite = reject; unknown on either side = neutral (0, no reject)</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Opposite carriageway -&gt; reject</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>x_cwz_connected</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Gate 3: proximity</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>The device is close enough to plausibly belong to the zone</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Distance to the zone geometry (snapped onto the line, or to the point) must be &lt;= 1600 m (~1 mi). Spatial credit = 25 * (1 - d/1600). &lt;= 150 m counts as effectively on the zone</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Beyond 1600 m -&gt; reject</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>x_connected_devices[].distanceM</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Gate 4: upstream (Field Escort rule)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>The board sits UPSTREAM of the zone in the served travel direction - traffic has not already passed it</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>isUpstream() against the matched reference point. Skipped when the device is alongside the zone or direction is unknown/BOTH</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Downstream -&gt; reject (it belongs to a different zone)</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>reasons[]</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Temporal</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>The device reported recently and inside the zone's active window</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Fresh = reported within 2 h (+5). Also checks the report timestamp falls between event start and end</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Stale still matches but scores 5 lower</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>fresh</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Deployment state</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>The board is actually ON, not blank / in transit</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>mode.displaying true (arrow/chevron/caution pattern) = +5</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>An off board can match but never AUTO-links (requireOnForAuto)</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>mode.displaying</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Scoring + banding</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Confidence is an honest number; questionable links go to a human</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>confidence = (40 if route known else 30) + dir + spatial + temporal + deploy. &gt;= 75 auto-link; 60-74 review queue; &lt; 60 no link. 'off' or &gt; 800 m block AUTO without lowering the score</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Below 60 no link; 60-74 surfaced for confirmation</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>x_connected_confidence</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>device-workzone-matcher.js DEFAULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DEVICE</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Independent post-check</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>The auto-links are audited using signals the matcher did NOT use</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Self-location parsed out of the device NAME ('SS2426 - I-35 NB @ MM 71.6') vs the feed's Route/Direction fields; message-vs-zone-type clash (the rest-area case); temporal; far / 'dir both' downgrades</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Link downgraded and surfaced in the validation panel</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>validation flags</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>device-validation.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - CAMERA</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Match (free, no network)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>There is a camera that could plausibly see the zone</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Nearest camera on the SAME interstate within 1500 m</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>No camera -&gt; no camera check is attempted</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>x_camera_id</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>camera-validation.js matchCamera</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - CAMERA</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Active-now gate</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Do not spend a vision call on a zone WZDx says is not running</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>isActiveNow(): now between start and end. null (no start date) also skips</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Skipped, no cost</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>camera-validation.js isActiveNow</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - CAMERA</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Vision inference</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Temporary traffic control is physically deployed, not stored</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>ONE inference on the still snapshot returning {work_zone, deployed, staged_only, devices[arrow-board,cones,barrels,drums,signs,workers,tma], confidence}. Only DEPLOYED counts - staged/stored cones do not</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>No detection = soft negative (proximity is not line-of-sight; most feeds have no PTZ/heading)</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>x_camera_verified, x_camera_detected</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>camera-validation.js detect</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - CAMERA</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Cost controls</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Vision spend cannot run away</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Gated on a vision key being set (otherwise available:false, $0); per-snapshot-URL cache TTL 10 min; on-demand only, never in a timer or the shared refresh; cheapest model, tiny token budget; max 25 zones per scan</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Silently unavailable rather than billing</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>camera-validation.js, camera-scan.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - CAMERA</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Check-count policy</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>A closure is never re-billed indefinitely</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Check #1 only within 90 min of start. If it sees nothing, ONE follow-up after 30 min. Hard cap 2 vision checks per closure ever. A non-detection while vision is off does NOT consume a check</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Ledger enforces the cap across restarts</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>camera_check_ledger.checks</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>camera-scan.js, camera-check-ledger.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - CAMERA</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Removal detection (daily)</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>A multi-day zone that is actually finished stops being elevated even if WZDx still lists it</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed multi-day closures get one check per 24 h; traffic control gone -&gt; tc_removed. This is the ONLY validator that can take verification away</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Zone drops out of the verified set</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>tc_removed</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>camera-check-ledger.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - PROBE (TomTom)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Category filter</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Only genuine work-zone incidents count as corroboration</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>iconCategory in {7 lane closed, 8 road closed, 9 road works}; lat/lon finite</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Other incident types ignored</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>tomtom-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - PROBE (TomTom)</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Spatial + route match</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>The independent incident is at the same place on the same road</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Same interstate, within 1500 m (maxM default)</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>No stamp applied</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>x_tomtom_corroborated</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>tomtom-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - PROBE (TomTom)</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Independence + cost</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>This is a genuinely non-DOT opinion, obtained cheaply</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>TomTom's own probe network, not the state that published the zone. Reuses the already-cached incident set - zero extra API calls in the corroborator. Upstream fetch is budget- and rate-capped with a circuit breaker</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Absence never demotes a zone</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>x_tomtom_corroborated</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>tomtom-corroboration.js, tomtom-incidents.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DMS</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Message content (strong)</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>The sign genuinely states roadwork or a closure</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>WZ_STRONG regex: ROAD WORK, WORK ZONE, LANE CLOSED, &lt;n&gt; LANES CLOSED, SHOULDER CLOSED/WORK, ROAD CLOSED, CLOSED AT/AHEAD/&lt;day&gt;, RAMP CLOSED, DETOUR, CONSTRUCTION, PAVING, MILLING, BRIDGE WORK, WORK AHEAD</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>No match -&gt; not evidence</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>x_dms_corroborated</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>dms-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - DMS</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Message content (exclusions)</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>The unrelated messages a board cycles through are never counted</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>WZ_EXCLUDE regex rejects Amber/Silver/Blue alerts, seat-belt / drive-sober / phone-down / move-over campaigns, travel times and '&lt;n&gt; MIN', weather (wind, fog, snow, ice), crashes and disabled vehicles, game-day traffic, election notices</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Rejected even if a STRONG token also appears</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>dms-corroboration.js isWorkZoneMsg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DMS</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Weak-token removal</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Bare tokens that also appear in incident and generic messages do not qualify</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Deliberately dropped from the old rule: a lone CLOSED, MERGE, WORKERS, REDUCED SPEED, EXPECT DELAY</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Requires a specific phrase instead</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>dms-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>4. Validator - DMS</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Spatial + route match</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>The sign is near the zone, on the same road when known</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Same interstate when known, within a few miles; zone must be active now</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>No stamp applied</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>x_dms_corroborated</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>dms-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>4. Validator - DMS</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Independence</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>A human operator in a different system posted this</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>DMS text is authored by an operator, not exported by the same automated WZDx pipeline being validated</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Absence never demotes</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>x_dms_corroborated</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>dms-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>5. Composition (CWZ 1.0)</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Positive-only semantics</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>A validator can only ever RAISE confidence</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>All four validators are positive-only. The single exception is the camera validator's daily removal check, which can withdraw verification</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Missing evidence is never treated as disproof</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>x_verification[]</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>cwz-roadevent-feed.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>5. Composition (CWZ 1.0)</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Source set</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Which independent systems agree about this zone</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>x_verification collects any of: device, camera, tomtom, dms</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Empty array = unverified</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>x_verification</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>cwz-roadevent-feed.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>5. Composition (CWZ 1.0)</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Corroboration count</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>How many INDEPENDENT sources agree - kept separate from how many devices are present</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>x_verification_count = number of distinct validators. x_connected_device_count is the physical device count and can be 0 while the zone is still corroborated by camera/TomTom/DMS</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>The two numbers are never conflated</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>x_verification_count</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>cwz-roadevent-feed.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>5. Composition (CWZ 1.0)</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Confidence tier</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Operator-facing banding of the corroboration count</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>&gt;= 2 sources = 'multi-source'; exactly 1 = 'single-source'; 0 = 'unverified'</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Drives the multi-source filter on the elevated feed</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>x_confidence_tier</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>cwz-roadevent-feed.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>5. Composition (CWZ 1.0)</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Sticky accumulation</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Evidence accumulates rather than flickering between refreshes</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Verification flags persist once earned (camera removal excepted), so a zone does not oscillate as individual sources come and go</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>x_connection_status</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>validation-ledger.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>5. Composition (CWZ 1.0)</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>WZDx output</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>The result is a spec-valid feed others can consume</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Emitted as WZDx v4.2 / CWZ 1.0 WorkZoneRoadEvent features with is_start_position_verified and the x_* evidence fields</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>full feature</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>cwz-roadevent-feed.js, cwz-device-feed.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>6. Monitoring</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Feed health</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>The upstream source itself is alive</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Is DMS_View returning data? how many devices are stale? fetch success history per feed</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Surfaced in the validation panel and availability dimension</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>device-validation.js, feed-tracking-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>6. Monitoring</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>How much of the network actually has independent evidence</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Share of active work zones with a connected device / any verification source</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Reported, not enforced</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>device-validation.js, coverage-gap-analyzer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>6. Monitoring</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Lifecycle</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Events are retired when they should be</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Event lifecycle manager ages out and closes events; camera tc_removed feeds the same decision</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Event leaves the active set</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>event-lifecycle-manager.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>6. Monitoring</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>Exceptions / stewardship</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>A human is told when something needs attention</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Work-zone exceptions raised to stewards (WZ_STEWARDS) via WZ_NOTIFY_WEBHOOK</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Notification</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>wz-exceptions.js</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G55"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add data-flow tab covering every dataset pulled and its use
"Data Pulled + How Used": 36 datasets across 24 domains, each with
source, extracted fields, refresh cadence, storage target, consuming
features, and which outbound feed it reaches. Covers work zones,
devices, cameras, probe traffic, weather, FARS crashes, IPAWS,
population, truck parking, geometry (ARNOLD/centerlines/RAMS), routing,
bridges/OSOW/border, major events, ITS assets, BIM/CADD, imagery,
grants, quality ledgers, collaboration, notifications, AI/ML, and
reference/platform data.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KU6vCHVwj8n3HqfggcJ2CP
</commit_message>
<xml_diff>
--- a/docs/Corridor_Communicator_API_Inventory.xlsx
+++ b/docs/Corridor_Communicator_API_Inventory.xlsx
@@ -8,22 +8,24 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal REST API" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Feed Registry" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External APIs Consumed" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Published Feeds" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera Sources" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DMS + Device Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Logic" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Pulled + How Used" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal REST API" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Feed Registry" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External APIs Consumed" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Published Feeds" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DMS + Device Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Logic" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Internal REST API'!$A$1:$I$512</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'State Feed Registry'!$A$1:$G$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'External APIs Consumed'!$A$1:$G$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Published Feeds'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Camera Sources'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DMS + Device Sources'!$A$1:$J$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Validation Logic'!$A$1:$G$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data Pulled + How Used'!$A$1:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Internal REST API'!$A$1:$I$512</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'State Feed Registry'!$A$1:$G$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'External APIs Consumed'!$A$1:$G$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Published Feeds'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Camera Sources'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DMS + Device Sources'!$A$1:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Validation Logic'!$A$1:$G$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +92,10 @@
       <b val="1"/>
       <color rgb="006B1F8C"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F6B78"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -135,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -201,6 +207,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -568,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2178,12 +2190,1791 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Data flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Data Pulled + How Used - every dataset ingested (36 across 24 domains): source, extracted fields, refresh cadence, storage, consumers, and which outbound feed it reaches</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>What we extract</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Refresh cadence</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Where it lands</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>How it is used</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Emitted in</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Implemented in</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Work zones</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>State work-zone events (WZDx v4.x / CWZ)</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>37 registered state feeds - see 'State Feed Registry'</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Event id, type, route, direction, start/end time, description, lanes affected, severity, geometry</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>On demand: 5-min cache, background refresh triggered at 4 min. No user-facing polling</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>eventsCache (in-process) + cached_events table with provenance, confidence_score, quality_flags, validation_status</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>The corridor map, /api/events, every validator's input set, DQI scoring, report cards</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>WZDx v4.2 feed, CWZ 1.0 RoadEvent feed, CIFS, TIM</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js, services/event-adapters.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Work zones</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Iowa lane-closure planning data</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Iowa DOT RoadClosures_public (AGOL, CORS-open)</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Planned closure geometry, route, dates</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>On demand when a builder opens</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Client-side in the builder (no backend hop)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Conflict check in the CARS 511 request builder - warns when a new request overlaps a planned closure</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>frontend builders (self-contained)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Work zones</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / fast-refresh feeds (Field Escort)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>purposebuiltsystems.github.io + registered plugin feeds</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Transient machine-published WZDx GeoJSON, expires_at</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Per-feed timer honoring plugin_data_feeds.refresh_interval (sub-hour)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>plugin_data_feeds tables, UPSERT by machine id, expired rows pruned</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Adds mobile/short-duration zones the hourly CIFS poller misses</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Flows into /api/events downstream</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>services/mobile-feed-ingest.js (draft, inert until wired in)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Devices</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>DMS + arrow board / portable sign feeds</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>18 state feeds - see 'DMS + Device Sources'</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Device id, type, portable flag, route, direction, coordinates, displayed message, mode.displaying, last updated</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Refreshed alongside the event cache (~5 min); Iowa DMS_View cached 10 min</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>devicesCache (roster + auto-links + review queue)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Device-to-work-zone auto-association (the strongest validator); DMS text corroboration; validation panel</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>CWZ 1.0 Device feed; x_cwz_connected / x_connected_devices on the RoadEvent feed</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>services/device-adapters.js, device-workzone-matcher.js, dms-corroboration.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Cameras</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Traffic camera inventory + still snapshots</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>15 state networks - see 'Camera Sources' (21,941 cameras)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Camera id, route, direction, milepost, coordinates, current still-image URL</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Inventory cached 30 min (locations are static); snapshots fetched only when a check is due</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>In-process camera cache; per-closure state in camera_check_ledger</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Camera-vision validation of whether traffic control is physically deployed; the daily removal check</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x_camera_verified / x_camera_detected / x_camera_url on the CWZ feed</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>services/camera-adapters.js, camera-validation.js, camera-scan.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Cameras</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Vision inference results</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Anthropic Messages API (or OpenAI / a self-hosted YOLO endpoint)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>{work_zone, deployed, staged_only, devices[arrow-board, cones, barrels, drums, signs, workers, tma], confidence}</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>One inference per due closure, max 2 per closure ever, 10-min per-snapshot cache, 25 zones per scan</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Elevation flags on the event + a training log (VISION_TRAINING_LOG on the Railway /data volume)</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Confirms deployed (not stored) traffic control; feeds the removal state machine</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>x_camera_* fields</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>services/camera-validation.js, vision-training-log.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Probe traffic</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>TomTom traffic incidents</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TomTom Traffic Incident Details v5</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Incident id, iconCategory (7 lane closed / 8 road closed / 9 road works), lat/lon, description</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Lazy: only polled when the layer is requested. Corridor TTL 45 min, zone-tile TTL 6 h (~800 req/day, self-capped at 2500)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>tomtomCache + tomtomZoneCache; validations banked in the validation ledger</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Independent non-DOT corroboration of work zones; the DOT-vs-consumer-nav deviation view</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>x_tomtom_corroborated</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>services/tomtom-incidents.js, tomtom-corroboration.js, tomtom-deviation.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>NWS active CAP alerts</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>https://api.weather.gov/alerts/active</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Alert id, event label, severity, urgency, certainty, areaDesc, derived state codes, geometry</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>On demand, cached</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>In-process cache</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Weather hazards on the corridor map; the single biggest gap-filler for the ~17 states with no public WZDx/511 feed; IPAWS context</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>/api/weather-alerts</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>services/nws-alerts.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>FARS historical crash records</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>NHTSA annual national CSV bundles (static.nhtsa.gov)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>accident.csv LATITUDE/LONGITUD, WRK_ZONE (0-4); vehicle.csv BODY_TYP large-truck range + MCARR_ID</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Monthly - scheduler runs on the 2nd at 4:00 AM. (The live CrashAPI 403s datacenter IPs, hence bulk files)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>crash_records in the PostGIS Postgres via crashDb (not the SQLite db)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Crash analytics: commercial-vehicle involvement and work-zone crashes clipped to within CRASH_CORRIDOR_BUFFER_MILES of the I-80 / I-35 polyline</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>/api/crashes/*</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>services/crash-data-service.js, scheduler-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>IPAWS / WEA alerting</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Iowa DOT IPAWS policy; 511ia.org + OSRM for geometry</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Qualifying closures (&gt;= 4 h or imminent danger), geofence polygons, CAP-XML payloads</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Evaluated against the active event set</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>ipaws_alert_log / ipaws_active_alerts (+ _lite variants)</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Automatic WEA qualification, precision geofence with population masking, multilingual CAP (EN/ES/Lao/Somali), audit log</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>/api/ipaws/* (33 endpoints)</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>services/ipaws-alert-service.js, ipaws-alert-service-lite.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Census population + urban extent</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Census decennial PL, TIGERweb, OSM Overpass/Nominatim, Google Earth Engine (LandScan)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Block-level population, urban area boundaries, POI/road context</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>On demand per geofence</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Computed per request; cached</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Population inside an IPAWS geofence, exclusion of populated/urban areas, real-time population-impact estimates for alert targeting</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>/api/population/*</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>services/population-density-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Truck parking</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>MAASTO TPIMS static + dynamic</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>8 Midwest DOTs via truckparking.travelmidwest.com (TPIMS V2.2), plus MnDOT IRIS, WisDOT transportal, TRIMARC</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Static: siteId, lat/lng, name, capacity, amenities. Dynamic: reportedAvailable, trend, open status. Joined on siteId</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Every 30 min (server timer)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>parking_facilities, parking_availability</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Live truck-parking availability on the map; ground truth for the prediction model</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>/api/parking/* (28 endpoints), /api/maasto-tpims</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>services/maasto-tpims.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Truck parking</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Iowa rest-area camera snapshots</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>atmsqf.iowadot.gov/snapshots/Public/RestAreas/*.jpg</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Still images of rest-area entrances, exits and truck-parking aprons</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Not stored; read at request time</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Visual occupancy check and calibration against the prediction model</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>/api/parking/*</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>truck_parking_service.js, services/parking-calibration-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Truck parking</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Historical occupancy patterns</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Derived internally from observations + bundled seed data</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Hour-of-week occupancy curves per facility, ground-truth observations, prediction accuracy</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Recomputed on demand; seeded at startup from bundled_data/truck_parking_patterns.json</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>parking_patterns, parking_occupancy_patterns, parking_observations, parking_ground_truth_observations, parking_prediction_accuracy</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Availability prediction where no live sensor exists; accuracy scoring of the predictions</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>/api/parking/*</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>parking_prediction.js, truck_parking_service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD linear-referenced road network</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>FHWA/BTS geo.dot.gov ARNOLD_&lt;ST&gt;_&lt;YEAR&gt; FeatureServers (48 mainland states)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Route polylines by route_id + milepost range</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>On demand per event needing geometry</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Enriched onto the event; osrm_geometry_cache / interstate_geometries</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Turns route+milepost work zones into real road-following linework instead of straight lines</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Geometry on every outbound feed</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>services/arnold-geometry-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>State centerlines + milepost layers</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Caltrans SHN, TxDOT Roadways/Mile Markers, NJ, IL, MO, WY, MA, CO ArcGIS services</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>State-native route ids and milepost points</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Enriched onto the event</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>State-centerline-first geometry - fixes the CA/TX case where ARNOLD route_id schemas do not match (CA uses name-composites, not '0005')</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Geometry on outbound feeds</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>services/state-centerline-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Iowa RAMS reference posts</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>gis.iowadot.gov Reference_Post_View</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Route, reference-post chainage</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>On demand, cached</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Iowa geometry cache (expired rows cleaned hourly)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Chainage-based linear position for device-to-work-zone matching, rather than raw straight-line distance</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>services/rams-chainage.js, iowa-geometry-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Routing</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>OSRM driving routes</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>router.project-osrm.org /route/v1/driving</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Route geometry (GeoJSON overview), distance, duration</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>On demand, queued and rate-limited</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>osrm_geometry_cache table (persisted so a route is never re-fetched)</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Detour and diversion-route generation, travel-time estimates, IPAWS geofence shaping</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>/api/diversion-routes/*, /api/osrm/*</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js, services/ipaws-alert-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Freight</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>National Bridge Inventory</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>NTAD NBI FeatureServer (services.arcgis.com/xOi1kZaI0eWDREZv)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Structure location, carries/crosses road names, vertical underclearance, NBI inspection date</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>On demand per work zone</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>bridge_clearances, bridge_clearance_warnings, bridge_restrictions</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>OSOW clearance layer; annotates any work zone with the structures the route passes UNDER (only those actually restrict you) plus a construction-proximity staleness flag</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Clearance fields on the DTCD / CWZ feed, /api/bridge-clearances/*</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>services/nbi-clearance.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Freight</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>CBP border wait times</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>https://bwt.cbp.gov/api/waittimes</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>port_number, port_name, crossing_name, border, hours, lane wait times (+ a locally maintained coordinate lookup, since CBP returns no lat/lng)</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>In-process cache</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Border crossings as map markers with live waits for freight corridor views; wait-time notifications</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>/api/border-wait-times, /api/border-notifications/*</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>services/border-wait-times.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Freight</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>State OSOW regulations + corridor regulations</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Curated / seeded reference content</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Per-state oversize-overweight rules, NASCO corridor regulations</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Seeded once at startup if empty (idempotent - manual edits survive redeploy)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>corridor_regulations, state OSOW tables</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Permit and routing guidance in the freight views</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>/api/state-osow-regulations/*, /api/corridor-regulations</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js, scripts/seed_corridor_regulations_if_empty.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Major events (concerts, games)</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Ticketmaster Discovery v2; PredictHQ as the alternate</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Event name, venue, coordinates, start time, expected attendance</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Cached 6 h; gated on the API key being set (Ticketmaster key not set yet)</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>majorEventsCache</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Demand-surge alerts near the corridor - warns when an event will load the same segment as a work zone</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>/api/major-events</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>services/ticketmaster-service.js, predicthq-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>ITS assets</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>ITS equipment + RSU inventory</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>NTAD RSU Deployment Locations; internally maintained equipment records</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Device type, location, status, health telemetry</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>its_equipment (3,149 rows), rsu_inventory, rsu_health, sensor_inventory (925), sensor_health, sensor_health_telemetry, device_health_snapshots</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>V2X / connected-vehicle layer, asset-health monitoring, predictive maintenance, network topology</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>/api/its-equipment/* (18), /api/v2x/*, /api/asset-health/*, /api/network/*</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>services/asset-health-monitor.js, predictive-maintenance-ai.js, device-health-store.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Digital infra</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>BIM / IFC models and CADD drawings</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>User-uploaded IFC, DXF and CADD files (+ buildingSMART schema references)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>IFC entities, DXF layers and entities, extracted geometry</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>On upload</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>ifc_models, cadd_models, cadd_layers, cadd_entities, infrastructure_elements, infrastructure_standards, infrastructure_gaps</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Digital-infrastructure inventory, standards crosswalk, gap analysis, GIS export of CADD content</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>/api/digital-infrastructure/* (12), /api/bim/*, /api/cadd/* (9)</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>services/cadd-processor.js, cadd-gis-exporter.js, dxf-extractor.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Imagery</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Aerial overlays</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>User-uploaded GeoTIFF / imagery</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Georeferenced raster tiles and bounds</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>On upload</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>S3-compatible object store (S3_ENDPOINT) + aerial_overlays metadata</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Aerial imagery overlay on the corridor map for planning and review</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>/api/aerial-overlays/*</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>services/aerial-overlays.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Grants</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Federal funding opportunities</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Grants.gov search2 + fetchOpportunity</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Opportunity number, title, agency, dates, eligibility, award ceiling - filtered by an ITS/digital-infrastructure keyword set (WZDx, connected corridors, CV/CAV, ITS deployment), NOT general transportation</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Grants tables</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Grant discovery, the proposal analyzer, and the grant package builder</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>/api/grants/* (23), /api/funding-opportunities/*</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>services/grants-service.js, compliance-analyzer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Feed fetch history and outcomes</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Recorded internally on every upstream fetch</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Success/failure, latency, record counts, per-feed timestamps</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Written on each fetch</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>quality_history, api_usage_logs, api_access_log, rate_limit_log</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>The Availability dimension of the DQI, feed outage detection, the state report cards</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>/api/data-quality/* (23), /api/reports/*, /api/quality/*</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>services/feed-tracking-service.js, feed-quality-scorer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Validation evidence ledger</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Produced by the four validators</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Per-zone verification sources, timestamps, confidence, sticky accumulation state</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>On each validation pass</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>validation ledger tables + camera_check_ledger</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Keeps verification from flickering between refreshes; supplies x_verification / x_confidence_tier</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>CWZ 1.0 feeds, /api/wz/*, /api/confidence/*</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>services/validation-ledger.js, camera-check-ledger.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Collaboration</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Coalition calendar, messages, community posts</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>User-generated in the platform</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Events, RSVPs, action items, artifacts, threads, reactions, biweekly reports</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>calendar_events, calendar_rsvps, calendar_action_items, calendar_artifacts, message_threads, message_reactions, alert_notifications</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>The I-80 coalition calendar, inter-state messaging, community board, biweekly reporting</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>/api/calendar/* (16), /api/messages/*, /api/community/*, /api/biweekly-reports/*</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>calendar-api.js, backend_proxy_server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Collaboration</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Vendor uploads</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Truck-parking and other vendor submissions</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Uploaded facility and availability data with provenance</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>On upload</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Vendor tables + parking tables</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Lets vendors contribute parking data where no state feed exists</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>/api/vendors/* (12)</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>vendor-upload-service.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Outbound alert delivery</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>SendGrid, Twilio, Slack, Microsoft Teams, ServiceNow</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Rendered alert payloads (email, SMS, webhook cards, incident tickets)</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>High-severity event check every 5 min; daily digest</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>alert_history, alert_rules, alerts</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Routing high-severity events and asset-health exceptions to the right people and systems</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>services/notification-service.js, email-service.js, daily-digest.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>LLM analysis and assistant</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Anthropic Messages API / OpenAI Chat Completions</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Prompts built from corridor data; structured JSON responses</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>On demand only - never on a shared or startup path</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>chat_conversations</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>The corridor briefing, NASCO corridor AI analysis, grant proposal analysis, the in-app assistant, and the custom-GPT action surface</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>/api/chat/*, /api/chatgpt/* (14), /api/corridor-briefing, /api/nasco-corridor-ai-analysis</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js, ml-integrations.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Prediction models</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Internal ML service (ML_SERVICE_URL, ml-service/)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Feature vectors from parking, event and traffic history</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Model outputs cached alongside the source tables</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Parking availability prediction, predictive maintenance, traffic-impact analysis</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>/api/ml/* (10), /api/predictive/*, /api/predictive-maintenance/*</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>ml-integrations.js, parking_prediction.js, traffic_impact_analyzer.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Interstate polylines (I-80, I-35)</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Loaded from PostGIS at startup</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Directional centerlines per corridor (i-80-eb/wb, i-35-nb/sb)</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Once at startup</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>interstatePolylinesCache, interstate_geometries</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Corridor clipping for crash data, geometry snapping, corridor analytics and the map base</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js getCorridorLine</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Interchanges and route restrictions</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Curated / admin-maintained</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Interchange locations, route restrictions</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Admin edits</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>interchanges, route_restrictions</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Detour feasibility, diversion routing, traveler information</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>/api/interchanges, /api/admin/interchanges</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Users, API keys, admin tokens</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Accounts, roles, hashed credentials, issued keys and their usage</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>users, api_keys, admin_tokens, api_access_log</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Authentication, state-level access control, API key issuance and rate limiting</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>/api/users/* (12), /api/admin/* (32)</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I37"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24043,7 +25834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25473,7 +27264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27199,7 +28990,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27510,7 +29301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28165,7 +29956,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29080,7 +30871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: break out connected arrow boards from portable DMS
The device tab conflated the two. Adding a live arrow-board count shows
66 total from only 2 states: Iowa 62 (Solar Tech / iCone AB units in
DMS_View) and Washington 4 (the one properly typed WZDx v4 Device Feed).
The other 4,654 devices are fixed or portable DMS, not arrow boards.

Also adds the Iowa DMS_View row, which was missing from the tab because
it is ingested via dms-corroboration.js / device-ingest.js rather than
the device-adapters registry.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KU6vCHVwj8n3HqfggcJ2CP
</commit_message>
<xml_diff>
--- a/docs/Corridor_Communicator_API_Inventory.xlsx
+++ b/docs/Corridor_Communicator_API_Inventory.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'External APIs Consumed'!$A$1:$G$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Published Feeds'!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Camera Sources'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'DMS + Device Sources'!$A$1:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'DMS + Device Sources'!$A$1:$K$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Validation Logic'!$A$1:$G$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,8 +98,9 @@
       <b val="1"/>
       <color rgb="000F6B78"/>
     </font>
+    <font/>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +125,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF6E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4EA"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,6 +255,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -616,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2283,6 +2295,41 @@
       <c r="A133" t="inlineStr">
         <is>
           <t>8 more device feeds unlock with a free 511 key: UT LA AZ NC NJ WI NV ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Connected arrow boards</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>66 arrow boards total, from only 2 states: Iowa 62 (DMS_View) and Washington 4 (WZDx v4 Device Feed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Every other device feed returns portable DMS, not arrow boards - 425 portable units across NY/PA/ME/OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Washington is the ONLY source with a properly typed device_type field; Iowa's are inferred from a device-name regex</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Vendor arrow-board fleets (iCone, Ver-Mac, HaulHub, Drivewyze) are not ingested directly - that is the MITRE partnership path</t>
         </is>
       </c>
     </row>
@@ -34669,22 +34716,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>State</t>
@@ -34717,863 +34765,916 @@
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
+          <t>ARROW BOARDS</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Portable DMS</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>Actively displaying</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Portable units</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Key required</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Iowa (DMS corroboration validator)</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Iowa DOT (DMS_View)</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>ArcGIS FeatureServer</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>https://services.arcgis.com/8lRhdTsQyJpO52F1/ArcGIS/rest/services/DMS_View/FeatureServer/0/query</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>not counted in this pull</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr"/>
-      <c r="G2" s="8" t="inlineStr"/>
-      <c r="H2" s="8" t="inlineStr"/>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="G2" s="35" t="n">
+        <v>62</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
-        <is>
-          <t>Primary DMS source for the DMS validator + device ingest; 10-min cache</t>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>The primary connected-device source. Arrow boards are Solar Tech - AB and iCone - AB units reporting real patterns (Right/Left Chevron sequential, Caution Four Corner flashing). NOTE: type is inferred from a NAME regex (/-\s*AB\b|arrow/i), not a typed field - a vendor naming a board differently is silently classed as DMS. Ingested via dms-corroboration.js / device-ingest.js, not device-adapters.js</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Arizona</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>CARS/OneStop 511</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>https://az511.com/api/v2/get/messagesigns</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>SKIPPED - no key</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr"/>
+      <c r="H3" s="8" t="inlineStr"/>
+      <c r="I3" s="8" t="inlineStr"/>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>Free key required</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>California</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Caltrans CWWP2 CMS (12 districts)</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>https://cwwp2.dot.ca.gov/data/d&lt;N&gt;/cms/cmsStatusD&lt;NN&gt;.json</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="5" t="n">
         <v>1016</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="I4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Some districts intermittently 500 and are skipped</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Florida</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>ArcGIS FeatureServer</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_MessageBoard/FeatureServer/0/query</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="8" t="n">
         <v>1047</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8" t="n">
         <v>520</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Fixed DMS with live message text</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Idaho</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>https://511.idaho.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Kentucky</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>ArcGIS FeatureServer</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>https://services2.arcgis.com/CcI36Pduqd0OR4W9/.../dmsSigns_2020/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>Fixed DMS with live message text</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Idaho</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Louisiana</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>CARS/OneStop 511</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>https://511.idaho.gov/api/v2/get/messagesigns</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>https://511la.org/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>SKIPPED - no key</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr"/>
-      <c r="G6" s="8" t="inlineStr"/>
-      <c r="H6" s="8" t="inlineStr"/>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Free key required</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Kentucky</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>ArcGIS FeatureServer</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>https://services2.arcgis.com/CcI36Pduqd0OR4W9/.../dmsSigns_2020/FeatureServer/0/query</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Maine</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>https://arcgisserver.maine.gov/arcgis/rest/services/mdot/MaineDOT_Dynamic/MapServer/111/query</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>83</v>
-      </c>
-      <c r="H7" s="5" t="n">
+      <c r="F9" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="G9" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H9" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Fixed DMS with live message text</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Louisiana</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Portable = trailer installation type</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Maryland</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer (CHART)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>https://chartimap1.sha.maryland.gov/arcgis/rest/services/CHART/DMS/MapServer/0/query</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>295</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>212</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Route/direction parsed from location string</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>CARS/OneStop 511</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>https://511la.org/api/v2/get/messagesigns</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nvroads.com/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>SKIPPED - no key</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr"/>
-      <c r="H8" s="8" t="inlineStr"/>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr"/>
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="K11" s="8" t="inlineStr">
         <is>
           <t>Free key required</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Maine</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>https://511nj.org/api/getmessagesigns</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>New Mexico</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Custom REST (NMRoads)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>https://servicev4.nmroads.com/RealMapWAR/GetMessageSigns</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>ERROR: certificate has expired</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>TLS certificate expired as of the pull</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511 (keyless path)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>https://511ny.org/api/getmessagesigns?format=json</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>919</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>919</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Keyless; 175 portable units detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>https://www.drivenc.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr"/>
+      <c r="I15" s="8" t="inlineStr"/>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Oklahoma</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Custom REST (oktraffic.org)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>https://oktraffic.org/api/Devices + /api/DmsStatuses</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>167</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>NTCIP MULTI tags stripped from message text</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>ArcGIS MapServer</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>https://arcgisserver.maine.gov/arcgis/rest/services/mdot/MaineDOT_Dynamic/MapServer/111/query</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>https://gis.penndot.gov/arcgis/rest/services/tsams/tsams/MapServer/17/query</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n">
-        <v>101</v>
-      </c>
-      <c r="G9" s="5" t="n">
+      <c r="F17" s="8" t="n">
+        <v>962</v>
+      </c>
+      <c r="G17" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="5" t="n">
-        <v>101</v>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="H17" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Portable = trailer installation type</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Maryland</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>ArcGIS MapServer (CHART)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>https://chartimap1.sha.maryland.gov/arcgis/rest/services/CHART/DMS/MapServer/0/query</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Portable = trailer / Type A-B structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Utah</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>CARS/OneStop 511</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.udottraffic.utah.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>SKIPPED - no key</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Free key required</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>WZDx v4 Device Feed</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>https://wzdx.wsdot.wa.gov/api/v4/DeviceFeed</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="F10" s="8" t="n">
-        <v>295</v>
-      </c>
-      <c r="G10" s="8" t="n">
-        <v>212</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="F19" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>Route/direction parsed from location string</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Nevada</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Only true WZDx device feed in the set - real arrow boards</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Wisconsin</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>CARS/OneStop 511</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.nvroads.com/api/v2/get/messagesigns</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>https://511wi.gov/api/v2/get/messagesigns</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>SKIPPED - no key</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Free key required</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>New Jersey</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>CARS/OneStop 511</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>https://511nj.org/api/getmessagesigns</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>SKIPPED - no key</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr"/>
-      <c r="H12" s="8" t="inlineStr"/>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Free key required</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>New Mexico</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Custom REST (NMRoads)</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>https://servicev4.nmroads.com/RealMapWAR/GetMessageSigns</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>ERROR: certificate has expired</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>TLS certificate expired as of the pull</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>CARS/OneStop 511 (keyless path)</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>https://511ny.org/api/getmessagesigns?format=json</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="n">
-        <v>919</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>919</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>175</v>
-      </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Keyless; 175 portable units detected</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>North Carolina</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>CARS/OneStop 511</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.drivenc.gov/api/v2/get/messagesigns</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>SKIPPED - no key</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Free key required</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Oklahoma</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Custom REST (oktraffic.org)</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>https://oktraffic.org/api/Devices + /api/DmsStatuses</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>167</v>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>51</v>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>NTCIP MULTI tags stripped from message text</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Pennsylvania</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>ArcGIS MapServer</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>https://gis.penndot.gov/arcgis/rest/services/tsams/tsams/MapServer/17/query</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>962</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>109</v>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Portable = trailer / Type A-B structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Utah</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>CARS/OneStop 511</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>https://www.udottraffic.utah.gov/api/v2/get/messagesigns</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>SKIPPED - no key</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr"/>
-      <c r="G18" s="8" t="inlineStr"/>
-      <c r="H18" s="8" t="inlineStr"/>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>Free key required</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Washington</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>WZDx v4 Device Feed</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>https://wzdx.wsdot.wa.gov/api/v4/DeviceFeed</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Only true WZDx device feed in the set - real arrow boards</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>WI</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Wisconsin</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>CARS/OneStop 511</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>https://511wi.gov/api/v2/get/messagesigns</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>SKIPPED - no key</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr"/>
-      <c r="G20" s="8" t="inlineStr"/>
-      <c r="H20" s="8" t="inlineStr"/>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Free key required</t>
-        </is>
-      </c>
-    </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr"/>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL (feeds that returned)</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr"/>
-      <c r="D21" s="18" t="inlineStr"/>
-      <c r="E21" s="18" t="inlineStr"/>
-      <c r="F21" s="18" t="n">
-        <v>4601</v>
-      </c>
-      <c r="G21" s="18" t="n">
-        <v>1789</v>
-      </c>
-      <c r="H21" s="18" t="n">
-        <v>429</v>
-      </c>
-      <c r="I21" s="18" t="inlineStr"/>
-      <c r="J21" s="18" t="inlineStr"/>
+      <c r="A21" s="17" t="inlineStr"/>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL (feeds returning data)</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr"/>
+      <c r="D21" s="17" t="inlineStr"/>
+      <c r="E21" s="17" t="inlineStr"/>
+      <c r="F21" s="17" t="n">
+        <v>4720</v>
+      </c>
+      <c r="G21" s="36" t="n">
+        <v>66</v>
+      </c>
+      <c r="H21" s="17" t="n">
+        <v>486</v>
+      </c>
+      <c r="I21" s="17" t="inlineStr"/>
+      <c r="J21" s="17" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J20"/>
+  <autoFilter ref="A1:K21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(device-adapters): surface Oklahoma's Trailer boards
ODOT's /api/DeviceTypeNames puts the DMS family under deviceTypeId 1
(Permanent / Portable / Lane Control / WeighStation) and models "Trailer"
as deviceTypeNameId 9 under its own deviceTypeId 4. None of the Trailer
units appear in /DmsStatuses — they carry no sign text — so they are
towable field boards, not message signs.

The adapter typed them 'dms' and did not flag them portable (isPortable
only checked deviceTypeNameId === 2), so all 10 were invisible to the
device↔work-zone matcher. Now typed 'arrow-board' and portable: 7 of the
10 surface (3 report 0,0 and are correctly dropped by normalize).

Brings the connected arrow-board total to 73 across IA (62), OK (7) and
WA (4). Matcher selftest passes; npm test passes.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KU6vCHVwj8n3HqfggcJ2CP
</commit_message>
<xml_diff>
--- a/docs/Corridor_Communicator_API_Inventory.xlsx
+++ b/docs/Corridor_Communicator_API_Inventory.xlsx
@@ -629,7 +629,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C139"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -657,6 +657,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -718,6 +719,7 @@
         <v>8</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -775,6 +777,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -2179,6 +2182,7 @@
         </is>
       </c>
     </row>
+    <row r="113"/>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
@@ -2214,6 +2218,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
@@ -2242,6 +2247,7 @@
         </is>
       </c>
     </row>
+    <row r="124"/>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
@@ -2256,6 +2262,7 @@
         </is>
       </c>
     </row>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
@@ -2298,6 +2305,7 @@
         </is>
       </c>
     </row>
+    <row r="134"/>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
@@ -2308,14 +2316,14 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>66 arrow boards total, from only 2 states: Iowa 62 (DMS_View) and Washington 4 (WZDx v4 Device Feed)</t>
+          <t>73 arrow boards total, from 3 states: Iowa 62 (DMS_View), Oklahoma 7 (Trailer class), Washington 4 (WZDx v4 Device Feed)</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Every other device feed returns portable DMS, not arrow boards - 425 portable units across NY/PA/ME/OK</t>
+          <t>Every other device feed returns portable or fixed DMS, not arrow boards - 486 portable DMS units across NY/PA/ME/OK</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2353,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -4404,7 +4412,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -6169,7 +6177,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I512"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -28029,7 +28037,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -29650,7 +29658,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -32025,7 +32033,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -33751,7 +33759,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -34062,7 +34070,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -34717,7 +34725,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -35450,11 +35458,11 @@
       <c r="F16" s="5" t="n">
         <v>167</v>
       </c>
-      <c r="G16" s="5" t="n">
-        <v>0</v>
+      <c r="G16" s="35" t="n">
+        <v>7</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>51</v>
@@ -35466,7 +35474,7 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>NTCIP MULTI tags stripped from message text</t>
+          <t>ODOT's /api/DeviceTypeNames models "Trailer" as deviceTypeNameId 9 under its own deviceTypeId 4 - a non-DMS field-device class, and none appear in /DmsStatuses (no sign text). 10 exist; 3 report 0,0 and are dropped. They carry no route, so the matcher infers it from the matched zone at reduced base credit. Fixed 2026-09-03 - previously typed 'dms' and not flagged portable, so all 10 were invisible.</t>
         </is>
       </c>
     </row>
@@ -35664,10 +35672,10 @@
         <v>4720</v>
       </c>
       <c r="G21" s="36" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="H21" s="17" t="n">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="I21" s="17" t="inlineStr"/>
       <c r="J21" s="17" t="inlineStr"/>

</xml_diff>